<commit_message>
[2026-07-27] 天策项目 - 修复C13列: 优先存储uuid(32位hex)而非token
</commit_message>
<xml_diff>
--- a/天策项目/2026-07-27/test_report_v25.xlsx
+++ b/天策项目/2026-07-27/test_report_v25.xlsx
@@ -820,12 +820,12 @@
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>178513808600050A32A69CRI7PMH9AXEC74</t>
+          <t>c72d6caf50f8449eaa7a32c33fec28bc</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
@@ -916,12 +916,12 @@
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>178513809100050A32A69QTJPF0HQC0032W</t>
+          <t>adffa9b282c14ea28fe8a4c3ae248e23</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
@@ -1013,12 +1013,12 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>178513809600050A32A69ROCQLXRNLJOUAK</t>
+          <t>b21f919f757840f89b4b3436f36dfec5</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>178513810100050A32A69LP5F8T8BHCXR6R</t>
+          <t>46a058dc4030431b80120ade7517b71e</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>178513810600050A32A69OAU3A8WHQEEFST</t>
+          <t>8c5f6978217443a9985dc6c0278bc5d7</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
@@ -1303,12 +1303,12 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>178513811100050A32A69P9XOJZ6DD1XJAW</t>
+          <t>afe555dcc6634ae1a99a92f49e52b44e</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -1400,12 +1400,12 @@
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>178513811600050A32A69E7FOPQUX7I4RYR</t>
+          <t>d7e5aa99db7d4dc3a1aed0fb16c08e09</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -1498,12 +1498,12 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>178513812100050A32A69H0OP0ZMR0O3F1M</t>
+          <t>060c7c8042b24f1cbcc799ebe3353e68</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
@@ -1597,12 +1597,12 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>178513812600050A32A69UKKZW7IBSWY6HU</t>
+          <t>1b1bda239ba0484cb911d35ae8d24aa1</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
@@ -1696,12 +1696,12 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>178513813100050A32A69QUESF8QG58VASI</t>
+          <t>579f8fdaa4d14d9e9e03f04b11ce7b2b</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
@@ -1794,12 +1794,12 @@
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>178513816500050A32A69DUTWHDHCF9C9NR</t>
+          <t>91d2edb3c2614faeba612982ead0391f</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
@@ -1893,12 +1893,12 @@
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>178513817000050A32A69DFK7GNNPRTIJG9</t>
+          <t>6bb8481aa1134a298e5d2d8422c0f739</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
@@ -1984,12 +1984,12 @@
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>178513817500050A32A69JUEPFANT6ZTUKR</t>
+          <t>cb55b3f1f58e4f1db710f3342cd707f8</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
@@ -2067,12 +2067,12 @@
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>178513818000050A32A69DKWUSWDA592GTC</t>
+          <t>1e093bfbf90642a5898bf33f136c6fd0</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>178513818500050A32A69AG30QHYQWOWHET</t>
+          <t>8daf1a6af9c544e5ae4e2462d642ddeb</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>178513819000050A32A69OVIEERRIRPKVPY</t>
+          <t>c8a27c74f7d9410ab1d456fdf981a864</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
@@ -2316,12 +2316,12 @@
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>178513819500050A32A69H6MSCKTL42TNQ8</t>
+          <t>63f57c89010949328942b874df706256</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
@@ -2399,12 +2399,12 @@
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>178513820000050A32A69JVGUXDEL5WX0KW</t>
+          <t>202bab7a659d4da3b94ac7b26ff8645e</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
@@ -2482,12 +2482,12 @@
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>178513820500050A32A69SMHR02EIJLYK3W</t>
+          <t>3da237bea31e46b8bffc47c2dfc9172b</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
@@ -2565,12 +2565,12 @@
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>178513821000050A32A69PGBRVMQNC9DQSJ</t>
+          <t>b8ac12c2381b4b3b9acc0808c534bcb8</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
@@ -2648,12 +2648,12 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>178513823000050A32A69HJVMI5LDTC4HYM</t>
+          <t>21672cd9c8e5467f9ae2cc92e984fc1e</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -2731,12 +2731,12 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>178513823500050A32A690AAOHBVQUK7UAV</t>
+          <t>537ccc4de0c14d73aab07b9d2063aadc</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -2814,12 +2814,12 @@
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>178513824000050A32A69R22XIFM8XKW2WM</t>
+          <t>f8ef34ee78dd4f8f8693143fa9164556</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
@@ -2897,12 +2897,12 @@
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>178513824500050A32A69XIX8WSRLXB2UKV</t>
+          <t>73466cba191443daada020522541d8f5</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>178513825000050A32A69PPRO3FAMQMSBHM</t>
+          <t>f462b684f02044488b6a0fcc6f27740b</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -3063,12 +3063,12 @@
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>178513825500050A32A698MH2J7SMXAQGAL</t>
+          <t>85eb8c8a90ac4c71af6607d6e607855d</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -3146,12 +3146,12 @@
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>178513826000050A32A690SELKSYV24DEMY</t>
+          <t>3f6fde6c8e424e5cbf2b73e2c23b5612</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
@@ -3229,12 +3229,12 @@
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>178513826500050A32A69OYWSO8G2BDSTZP</t>
+          <t>b37cb4c9020b4b078580f01572a994eb</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr">
@@ -3312,12 +3312,12 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>178513827000050A32A69BASM3MWHWSPN31</t>
+          <t>3f6e6850714a4cee91db68d679d1e316</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
@@ -3395,12 +3395,12 @@
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>178513827500050A32A69RLH3XMIU2JISIF</t>
+          <t>a5fa94a6f6ca478aad4e5167660e231e</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr">
@@ -3478,12 +3478,12 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>178513831800050A32A69TB4ASTGHHC7ZQP</t>
+          <t>0558e6eacbaf44289a75163565757c94</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
@@ -3563,12 +3563,12 @@
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>178513832300050A32A69GJQQHIRSFRYUDS</t>
+          <t>3431709142b54a349e688a54ba4f8dff</t>
         </is>
       </c>
       <c r="N33" s="4" t="inlineStr">
@@ -3648,12 +3648,12 @@
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>178513832800050A32A69MX3BKBLJOBR6EM</t>
+          <t>1c7f10af519e41e6b96d39a164b600bc</t>
         </is>
       </c>
       <c r="N34" s="4" t="inlineStr">
@@ -3733,12 +3733,12 @@
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
-          <t>178513833300050A32A69TLN6TRXMB7FOOK</t>
+          <t>b720bd5ec9ba472b95dbafc59b1acf22</t>
         </is>
       </c>
       <c r="N35" s="4" t="inlineStr">
@@ -3816,12 +3816,12 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>178513833800050A32A69BV1N2SWSP8OULI</t>
+          <t>49450452e9ac4e57aaa7087173a71d47</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -3905,12 +3905,12 @@
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>178513834300050A32A6914E1NE5USNDMJI</t>
+          <t>b556f7570566450e90c5ac6c25a64598</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -4001,12 +4001,12 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>178513834800050A32A69UGQOR42JRDF58T</t>
+          <t>47bc3c0cb1cc4f0f96c8f5e8e09b24ef</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
@@ -4097,12 +4097,12 @@
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>178513835300050A32A69KQE8GY0DD3JRAQ</t>
+          <t>a7ee294ad69c495787906a09bdcfb3d6</t>
         </is>
       </c>
       <c r="N39" s="4" t="inlineStr">
@@ -4193,12 +4193,12 @@
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>178513835800050A32A69IO415C9WPH7PJS</t>
+          <t>27a87e997a244be5b6c983491e2ea4fd</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
@@ -4289,12 +4289,12 @@
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>178513836300050A32A69CKBNFFWAOZLX8C</t>
+          <t>2dd6d388b5a94ca4965809a47b4e86c0</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
@@ -4386,12 +4386,12 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>178513841000050A32A69DNC8VREDGS28BD</t>
+          <t>d350d491f9a540b5a7b3b60b456b38b9</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
@@ -4483,12 +4483,12 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>178513841500050A32A69UEFTJYHFXMWOYH</t>
+          <t>f4762197dcd5432fbfcb6c2f58e0f146</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -4580,12 +4580,12 @@
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M44" s="4" t="inlineStr">
         <is>
-          <t>178513842000050A32A69KJ7FMXGVW3EPBY</t>
+          <t>eb14d8bdfe744853a539b4082380e32e</t>
         </is>
       </c>
       <c r="N44" s="4" t="inlineStr">
@@ -4677,12 +4677,12 @@
       </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>178513842500050A32A69JYQZGZVUKPVUIU</t>
+          <t>37b4a581190b4062ad365057cb82d523</t>
         </is>
       </c>
       <c r="N45" s="4" t="inlineStr">
@@ -4774,12 +4774,12 @@
       </c>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
         <is>
-          <t>178513843000050A32A69KCA9CPYIBGOFIZ</t>
+          <t>fb5d03f3efdf4efa80837a4cc067d973</t>
         </is>
       </c>
       <c r="N46" s="4" t="inlineStr">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr">
@@ -5039,7 +5039,7 @@
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M58" s="4" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M59" s="4" t="inlineStr">
@@ -5996,7 +5996,7 @@
       </c>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="L62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M62" s="4" t="inlineStr">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M63" s="4" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="L64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M64" s="4" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M65" s="4" t="inlineStr">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M66" s="4" t="inlineStr">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="L67" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M67" s="4" t="inlineStr">
@@ -6692,7 +6692,7 @@
       </c>
       <c r="L68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M68" s="4" t="inlineStr">
@@ -6779,7 +6779,7 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
@@ -6866,7 +6866,7 @@
       </c>
       <c r="L70" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:43</t>
+          <t>2026-07-28 16:19</t>
         </is>
       </c>
       <c r="M70" s="4" t="inlineStr">

</xml_diff>